<commit_message>
verifier_architecture : écart sans valeur attendue, tolérance 7 cm justifiée, fixture synthétique, M23-M25 non nommés (E-187 mini-lot 1)
</commit_message>
<xml_diff>
--- a/seances/0b/DeepCwind_ARCHITECTURE.xlsx
+++ b/seances/0b/DeepCwind_ARCHITECTURE.xlsx
@@ -3232,11 +3232,6 @@
           <t>M23</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Base column cap 1</t>
-        </is>
-      </c>
       <c r="C24" t="inlineStr">
         <is>
           <t>Bases</t>
@@ -3269,11 +3264,6 @@
           <t>M24</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Base column cap 2</t>
-        </is>
-      </c>
       <c r="C25" t="inlineStr">
         <is>
           <t>Bases</t>
@@ -3304,11 +3294,6 @@
       <c r="A26" t="inlineStr">
         <is>
           <t>M25</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Base column cap 3</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">

</xml_diff>